<commit_message>
Tighten terminal-value margins after audit (SNOW 18%->15%, NTNX 17%->16%)
Re-derived every terminal uFCF margin from its stated steady-state logic
(EBIT x (1-tax) + D&A - capex - g x NWC). SNOW's 18% was ~6pts above its
own Investor-Day-glidepath derivation (~12%); reset to the 15% midpoint of
a documented 12-18% band. NTNX trimmed to the derived 16%. Mid-year
perpetuity discounting verified exact (brute-force check); ReadMe now
documents the reconciliation identity.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0187dABUdEhW8gT5WAkj3Fgw
</commit_message>
<xml_diff>
--- a/dcf/dcf_models.xlsx
+++ b/dcf/dcf_models.xlsx
@@ -285,7 +285,7 @@
     <t xml:space="preserve">Normalized terminal uFCF margin (× yr-5 revenue)</t>
   </si>
   <si>
-    <t xml:space="preserve">steady state: ~28% non-GAAP OM − ~10% SBC, taxed, + deferred-rev inflow</t>
+    <t xml:space="preserve">derived: 18% steady-state econ EBIT (28% NG OM − 10% SBC) × 0.8 tax = 14.4% + ~1.2pt deferred-rev inflow &amp; D&amp;A&gt;capex</t>
   </si>
   <si>
     <t xml:space="preserve">Terminal uFCF (yr-5 revenue × (1+g) × margin)</t>
@@ -336,7 +336,7 @@
     <t xml:space="preserve">Growth: FY26 guide $2.82–2.84B (+11.5%) accelerating toward management's 'mid-to-high-teens by FY2029' framework (Q3 FY26 call, May 27, 2026) on VMware/Broadcom displacement; ARR $2.43B +15%. Sept-2023 investor-day $3B-ARR-by-FY27 target looks late by ~a year on the new ARR methodology.</t>
   </si>
   <si>
-    <t xml:space="preserve">Margins: FY26 non-GAAP op margin ~22.5% guided, but SBC is ~13% of revenue — economic EBIT starts ~10% and scales to 18% as SBC leverage improves. FCF guide $760–780mm (~27%) is before SBC; to replicate a street-style model set margins to 22.5%→28%. ΔNWC −20% of Δrev captures the deferred-revenue cash inflow of the subscription model.</t>
+    <t xml:space="preserve">Margins: FY26 non-GAAP op margin ~22.5% guided, but SBC is ~13% of revenue — economic EBIT starts ~10% and scales to 18% as SBC leverage improves. FCF guide $760–780mm (~27%) is before SBC; to replicate a street-style model set margins to 22.5%→28% (lifts the DCF to ≈$60, near today's price). ΔNWC −20% of Δrev captures the deferred-revenue cash inflow of the subscription model.</t>
   </si>
   <si>
     <t xml:space="preserve">Net cash treats both converts as debt while using the diluted share count (conservative double-count on the ITM 2027 notes). $750mm buyback authorization added May 2026 not modeled.</t>
@@ -405,13 +405,13 @@
     <t xml:space="preserve">normalized; large NOLs defer cash taxes</t>
   </si>
   <si>
-    <t xml:space="preserve">steady state: ~30% non-GAAP OM − ~15% SBC, taxed, + deferred-rev inflow</t>
+    <t xml:space="preserve">band 12–18%: Investor-Day glidepath (30% NG OM − 15% SBC, taxed, + inflows) derives ~12%; 18% needs ~35% NG OM at scale. Base = midpoint 15%</t>
   </si>
   <si>
     <t xml:space="preserve">Growth: FY27 product guide $5.84B +31% (raised May 27, 2026; Q1 product +34%, NRR 126%, RPO $9.2B +38%). Path hits ~$10B product revenue in FY2030 — one year later than the FY29 target reaffirmed at the Jun 2, 2026 Investor Day (management framed FY29 $10B as 'worst case'; this model is slightly more conservative). $6B/5-yr AWS pact, Observe deal.</t>
   </si>
   <si>
-    <t xml:space="preserve">Margins: the SBC problem dominates — SBC still ~29% of revenue (down from 41% FY25; Investor Day glidepath to 27%, assumed to keep falling). Economic EBIT is negative until ~FY2029, consistent with the Investor Day commitment of GAAP profitability by Q4 FY28. Non-GAAP op margin 13.5% and adj FCF margin ~23–25% guided for FY27 — a street-style model (margins 13.5%→28%) roughly triples the DCF value; that is the entire bull/bear debate on SNOW.</t>
+    <t xml:space="preserve">Margins: the SBC problem dominates — SBC still ~29% of revenue (down from 41% FY25; Investor Day glidepath to 27%, assumed to keep falling). Economic EBIT is negative until ~FY2029, consistent with the Investor Day commitment of GAAP profitability by Q4 FY28. Non-GAAP op margin 13.5% and adj FCF margin ~23–25% guided for FY27 — a street-style model (explicit margins 13.5%→28%, terminal 25%) roughly doubles the DCF value to ~$115, still ~65% below the price; that is the entire bull/bear debate on SNOW.</t>
   </si>
   <si>
     <t xml:space="preserve">ΔNWC −15% of Δrev captures the strong deferred-revenue/prepaid-consumption cash cycle.</t>
@@ -753,7 +753,7 @@
     <t xml:space="preserve">• Mid-year discounting convention (periods 0.5 … 4.5). For companies whose fiscal year 1 is already partly elapsed (Jan/Feb/Jun/Jul FYE), this slightly flatters PV; immaterial to conclusions.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Terminal value: Gordon growth on a NORMALIZED terminal uFCF margin × year-5 revenue. For the cyclical memory names (SK hynix, Samsung, Sandisk, Kioxia) the terminal margin is set near MID-CYCLE, not the current super-cycle peak, so the perpetuity does not capitalize peak earnings. For the software names it is set at estimated steady-state economics rather than the year-5 point on the transition path.</t>
+    <t xml:space="preserve">• Terminal value: Gordon growth on a NORMALIZED terminal uFCF margin × year-5 revenue. For the cyclical memory names (SK hynix, Samsung, Sandisk, Kioxia) the terminal margin is set near MID-CYCLE, not the current super-cycle peak, so the perpetuity does not capitalize peak earnings. For the software names it is set at estimated steady-state economics rather than the year-5 point on the transition path. Each margin reconciles as: steady-state economic EBIT × (1−tax) + D&amp;A − capex − growth×NWC (the derivation is on each tab). Discounting is mid-year-consistent: PV(TV) = [TFCF/(WACC−g)] × DF(4.5) is the exact value of a perpetuity whose payments land at mid-year, matching the explicit period.</t>
   </si>
   <si>
     <t xml:space="preserve">• Net cash = latest-quarter cash + investments − total debt (incl. converts). Diluted shares = latest reported diluted count; future buybacks and dilution are not separately modeled.</t>
@@ -1536,11 +1536,11 @@
       </c>
       <c r="E5" s="7" t="n">
         <f aca="false">NTNX!B48</f>
-        <v>41.4635330747409</v>
+        <v>39.6371847059448</v>
       </c>
       <c r="F5" s="8" t="n">
         <f aca="false">NTNX!B50</f>
-        <v>-0.384357341132281</v>
+        <v>-0.411474614611065</v>
       </c>
       <c r="G5" s="8" t="n">
         <f aca="false">POWER(NTNX!G15/NTNX!B15,1/5)-1</f>
@@ -1560,11 +1560,11 @@
       </c>
       <c r="K5" s="8" t="n">
         <f aca="false">NTNX!B35</f>
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="L5" s="8" t="n">
         <f aca="false">NTNX!B45</f>
-        <v>0.792416785697453</v>
+        <v>0.782267683189855</v>
       </c>
       <c r="M5" s="9" t="s">
         <v>18</v>
@@ -1636,11 +1636,11 @@
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">SNOW!B48</f>
-        <v>72.1001998709608</v>
+        <v>61.2947426707697</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">SNOW!B50</f>
-        <v>-0.778636824564917</v>
+        <v>-0.811811910378037</v>
       </c>
       <c r="G7" s="8" t="n">
         <f aca="false">POWER(SNOW!G15/SNOW!B15,1/5)-1</f>
@@ -1660,11 +1660,11 @@
       </c>
       <c r="K7" s="8" t="n">
         <f aca="false">SNOW!B35</f>
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="L7" s="8" t="n">
         <f aca="false">SNOW!B45</f>
-        <v>0.955052130276908</v>
+        <v>0.946543110988904</v>
       </c>
       <c r="M7" s="9" t="s">
         <v>21</v>
@@ -4015,7 +4015,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="54" t="s">
         <v>240</v>
       </c>
@@ -4646,7 +4646,7 @@
         <v>83</v>
       </c>
       <c r="B35" s="20" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>84</v>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="B36" s="28" t="n">
         <f aca="false">G15*(1+$B$10)*B35</f>
-        <v>957.810431019235</v>
+        <v>901.46864095928</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="B37" s="28" t="n">
         <f aca="false">B36/($B$9-$B$10)</f>
-        <v>13683.0061574176</v>
+        <v>12878.1234422754</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4676,7 +4676,7 @@
       </c>
       <c r="B38" s="28" t="n">
         <f aca="false">B37*G31</f>
-        <v>8910.75369135633</v>
+        <v>8386.59170951184</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4685,7 +4685,7 @@
       </c>
       <c r="B39" s="34" t="n">
         <f aca="false">B37/G27</f>
-        <v>14.2867785306325</v>
+        <v>13.4463797935365</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="B43" s="28" t="n">
         <f aca="false">B38</f>
-        <v>8910.75369135633</v>
+        <v>8386.59170951184</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="B44" s="25" t="n">
         <f aca="false">B42+B43</f>
-        <v>11245.0339924506</v>
+        <v>10720.8720106061</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="B45" s="30" t="n">
         <f aca="false">B43/B44</f>
-        <v>0.792416785697453</v>
+        <v>0.782267683189855</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="B47" s="25" t="n">
         <f aca="false">B44+B46</f>
-        <v>11900.0339924506</v>
+        <v>11375.8720106061</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="B48" s="35" t="n">
         <f aca="false">B47*$B$11/B6</f>
-        <v>41.4635330747409</v>
+        <v>39.6371847059448</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="B50" s="37" t="n">
         <f aca="false">B48/B49-1</f>
-        <v>-0.384357341132281</v>
+        <v>-0.411474614611065</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4823,23 +4823,23 @@
       </c>
       <c r="C54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B54-C$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>42.6657678585489</v>
+        <v>40.7812753705021</v>
       </c>
       <c r="D54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B54-D$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>45.2992253097938</v>
+        <v>43.259823559909</v>
       </c>
       <c r="E54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B54-E$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>48.3715923362462</v>
+        <v>46.1514631142172</v>
       </c>
       <c r="F54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B54-F$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>52.0025715493263</v>
+        <v>49.5688553147632</v>
       </c>
       <c r="G54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B54-G$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>56.3597466050224</v>
+        <v>53.6697259554183</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4849,23 +4849,23 @@
       </c>
       <c r="C55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B55-C$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>39.812511679201</v>
+        <v>38.0895052750003</v>
       </c>
       <c r="D55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B55-D$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>42.0585735989625</v>
+        <v>40.2034459053641</v>
       </c>
       <c r="E55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B55-E$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>44.6501835063797</v>
+        <v>42.6426081711685</v>
       </c>
       <c r="F55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B55-F$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>47.6737283983664</v>
+        <v>45.4882974812737</v>
       </c>
       <c r="G55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B55-G$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>51.2470087252598</v>
+        <v>48.8513848477616</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4875,23 +4875,23 @@
       </c>
       <c r="C56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B56-C$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>37.3187861698273</v>
+        <v>35.7362464424967</v>
       </c>
       <c r="D56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B56-D$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>39.2530013921203</v>
+        <v>37.5566842987725</v>
       </c>
       <c r="E56" s="41" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B56-E$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>41.4635330747409</v>
+        <v>39.6371847059448</v>
       </c>
       <c r="F56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B56-F$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>44.0141465546877</v>
+        <v>42.0377620988359</v>
       </c>
       <c r="G56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B56-G$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>46.9898622812923</v>
+        <v>44.8384357238755</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4901,23 +4901,23 @@
       </c>
       <c r="C57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B57-C$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>35.1210868647821</v>
+        <v>33.6617266088555</v>
       </c>
       <c r="D57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B57-D$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>36.800871326031</v>
+        <v>35.2427002194427</v>
       </c>
       <c r="E57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B57-E$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>38.7046270487797</v>
+        <v>37.0344703114415</v>
       </c>
       <c r="F57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B57-F$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>40.8803478747782</v>
+        <v>39.0822075594401</v>
       </c>
       <c r="G57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B57-G$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>43.3907949816996</v>
+        <v>41.4449813071308</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4927,23 +4927,23 @@
       </c>
       <c r="C58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B58-C$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>33.1700228106463</v>
+        <v>31.8194569193149</v>
       </c>
       <c r="D58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B58-D$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>34.6397562806246</v>
+        <v>33.2027354792945</v>
       </c>
       <c r="E58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B58-E$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>36.2932064343501</v>
+        <v>34.7589238592714</v>
       </c>
       <c r="F58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B58-F$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>38.1671166085724</v>
+        <v>36.5226040232454</v>
       </c>
       <c r="G58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B58-G$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>40.308728236255</v>
+        <v>38.5382384963584</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6548,7 +6548,7 @@
         <v>83</v>
       </c>
       <c r="B35" s="20" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>124</v>
@@ -6560,7 +6560,7 @@
       </c>
       <c r="B36" s="28" t="n">
         <f aca="false">G15*(1+$B$10)*B35</f>
-        <v>2631.6274817065</v>
+        <v>2193.02290142208</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6569,7 +6569,7 @@
       </c>
       <c r="B37" s="28" t="n">
         <f aca="false">B36/($B$9-$B$10)</f>
-        <v>37594.6783100928</v>
+        <v>31328.898591744</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="B38" s="28" t="n">
         <f aca="false">B37*G31</f>
-        <v>23988.1149844242</v>
+        <v>19990.0958203535</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="B39" s="34" t="n">
         <f aca="false">B37/G27</f>
-        <v>25.3998294615561</v>
+        <v>21.1665245512967</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6616,7 +6616,7 @@
       </c>
       <c r="B43" s="28" t="n">
         <f aca="false">B38</f>
-        <v>23988.1149844242</v>
+        <v>19990.0958203535</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6625,7 +6625,7 @@
       </c>
       <c r="B44" s="25" t="n">
         <f aca="false">B42+B43</f>
-        <v>25117.0739522555</v>
+        <v>21119.0547881848</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="B45" s="30" t="n">
         <f aca="false">B43/B44</f>
-        <v>0.955052130276908</v>
+        <v>0.946543110988904</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="B47" s="25" t="n">
         <f aca="false">B44+B46</f>
-        <v>26677.0739522555</v>
+        <v>22679.0547881848</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6661,7 +6661,7 @@
       </c>
       <c r="B48" s="35" t="n">
         <f aca="false">B47*$B$11/B6</f>
-        <v>72.1001998709608</v>
+        <v>61.2947426707697</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="B50" s="37" t="n">
         <f aca="false">B48/B49-1</f>
-        <v>-0.778636824564917</v>
+        <v>-0.811811910378037</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6725,23 +6725,23 @@
       </c>
       <c r="C54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B54-C$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>74.3143921292827</v>
+        <v>63.1664840805736</v>
       </c>
       <c r="D54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B54-D$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>79.8109591746876</v>
+        <v>67.7469566184109</v>
       </c>
       <c r="E54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B54-E$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>86.2236207276599</v>
+        <v>73.0908412458878</v>
       </c>
       <c r="F54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B54-F$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>93.802220744809</v>
+        <v>79.4063412601788</v>
       </c>
       <c r="G54" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B54,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B54-G$53)/POWER(1+$B54,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>102.896540765388</v>
+        <v>86.9849412773279</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6751,23 +6751,23 @@
       </c>
       <c r="C55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B55-C$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>68.5077088266104</v>
+        <v>58.3141318327727</v>
       </c>
       <c r="D55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B55-D$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>73.1960438899782</v>
+        <v>62.2210777189126</v>
       </c>
       <c r="E55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B55-E$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>78.6056612707873</v>
+        <v>66.7290922029201</v>
       </c>
       <c r="F55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B55-F$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>84.9168815483978</v>
+        <v>71.9884424342623</v>
       </c>
       <c r="G55" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B55,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B55-G$53)/POWER(1+$B55,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>92.3755964219375</v>
+        <v>78.204038162212</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6777,23 +6777,23 @@
       </c>
       <c r="C56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B56-C$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>63.4480040693585</v>
+        <v>54.0845795027678</v>
       </c>
       <c r="D56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B56-D$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>67.4856954434396</v>
+        <v>57.449322314502</v>
       </c>
       <c r="E56" s="41" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B56-E$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>72.1001998709608</v>
+        <v>61.2947426707697</v>
       </c>
       <c r="F56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B56-F$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>77.4246280565622</v>
+        <v>65.7317661587709</v>
       </c>
       <c r="G56" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B56,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B56-G$53)/POWER(1+$B56,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>83.6364609397638</v>
+        <v>70.9082935614389</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6803,23 +6803,23 @@
       </c>
       <c r="C57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B57-C$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>59.0029399656757</v>
+        <v>50.3675366925798</v>
       </c>
       <c r="D57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B57-D$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>62.5097561729208</v>
+        <v>53.2898835319507</v>
       </c>
       <c r="E57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B57-E$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>66.4841478744652</v>
+        <v>56.601876616571</v>
       </c>
       <c r="F57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B57-F$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>71.0263098190873</v>
+        <v>60.3870115704228</v>
       </c>
       <c r="G57" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B57,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B57-G$53)/POWER(1+$B57,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>76.267265909036</v>
+        <v>64.7544749787133</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6829,23 +6829,23 @@
       </c>
       <c r="C58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+C$53)*$B$35/($B58-C$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>55.0696022499099</v>
+        <v>47.077232976372</v>
       </c>
       <c r="D58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+D$53)*$B$35/($B58-D$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>58.1381216438823</v>
+        <v>49.634332471349</v>
       </c>
       <c r="E58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+E$53)*$B$35/($B58-E$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>61.5902059621013</v>
+        <v>52.5110694031981</v>
       </c>
       <c r="F58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+F$53)*$B$35/($B58-F$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>65.5025681894161</v>
+        <v>55.7713712592938</v>
       </c>
       <c r="G58" s="40" t="n">
         <f aca="false">(SUMPRODUCT($C$27:$G$27,1/POWER(1+$B58,$C$30:$G$30))+$G$15*(1+G$53)*$B$35/($B58-G$53)/POWER(1+$B58,$G$30)+$B$7)*$B$11/$B$6</f>
-        <v>69.9738393063473</v>
+        <v>59.4974305234031</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>